<commit_message>
Update documentation for 1.9.0 and strip personal metadata from docs
Documentation
- capability-modbus-mapping.md: poll groups, new capabilities and flow
  cards, fault bit fields, on/off via 4-2101, dynamic setpoint limits;
  correct measure_power (always Modbus) and measure_water entries
- building-model-sample-gating.md: add the blocked_dhw_active gate
- setup README and port setting hint: port must match the gateway's
  Local port (guide uses 502, EW11A default 8899), serial protocol Modbus
- CLAUDE.md, AGENTS.md, GEMINI.md: unit tests via npm test, poll-group
  snapshots, current dashboard pages

Metadata
- Remove absolute save paths and author names from the metadata of the
  .xlsx files under docs/ (cell content unchanged)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014bZY8mkkHE18TKcc3FjQ54
</commit_message>
<xml_diff>
--- a/docs/Heatpump specs/modbus/Adlar III/HHi/Adlar-III_modbus_registers HHi.xlsx
+++ b/docs/Heatpump specs/modbus/Adlar III/HHi/Adlar-III_modbus_registers HHi.xlsx
@@ -3,11 +3,6 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hermanhilberink/Documents/privé/warmtepomp/handleidingen/modbus/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{86332D90-4103-AF45-AFB4-36FE716C045F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="60" yWindow="0" windowWidth="33920" windowHeight="28800" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>

</xml_diff>